<commit_message>
use of medication fix
</commit_message>
<xml_diff>
--- a/SurveyQuestions/csvs/hms_survey.xlsx
+++ b/SurveyQuestions/csvs/hms_survey.xlsx
@@ -3428,7 +3428,7 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>1=YourDost 2=Urgent Care or the Emergency Room 3=Provider in the local community (not on campus) 4=Provider in my hometown 5=Provider affiliated with a telehealth company 6=Others</t>
+          <t>1=YourDost 2=Urgent Care or the Emergency Room 3=Provider in the local community (not on campus) 4=Provider in my hometown 5=Provider affiliated with a telehealth company 6=Other (please specify)</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Display if "1=Attention deficit hyperactivity disorder (ADHD or ADD)" is selected for "Specifically, which of the following neurodevelopmental disorder or intellectual disability were you diagnosed with by a professional? (Select all that apply)"</t>
+          <t>Display if "1=Attention deficit hyperactivity disorder (ADHD or ADD)" is selected for "Specifically, which of the following neurodevelopmental disorder or intellectual disability were you diagnosed with by a professional? (Select all that apply)" or "1=Attention deficit/hyperactivity disorders" is selected for "Do you have a disability or disabilities from any of the following categories?"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
use of meds fix #2
</commit_message>
<xml_diff>
--- a/SurveyQuestions/csvs/hms_survey.xlsx
+++ b/SurveyQuestions/csvs/hms_survey.xlsx
@@ -3352,7 +3352,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?”</t>
+          <t>Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?” Display if “8=No, none of these” is not selected for “In the past 12 months have you taken any of the following types of prescription medications?”</t>
         </is>
       </c>
     </row>
@@ -3487,7 +3487,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?”</t>
+          <t>Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?” Display if “8=No, none of these” is not selected for “In the past 12 months have you taken any of the following types of prescription medications?”</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
changed financing edu section
</commit_message>
<xml_diff>
--- a/SurveyQuestions/csvs/hms_survey.xlsx
+++ b/SurveyQuestions/csvs/hms_survey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Demographics" sheetId="1" state="visible" r:id="rId3"/>
@@ -1346,13 +1346,13 @@
     <t xml:space="preserve">Display if “Yes” is selected for “Do you have any concerns about your current living situation, like housing conditions, safety, and costs?”</t>
   </si>
   <si>
+    <t xml:space="preserve">Financing education</t>
+  </si>
+  <si>
     <t xml:space="preserve">Which of the following have you used to pay for educational expenses (room, board, tuition, and fees)? (Select all that apply)</t>
   </si>
   <si>
     <t xml:space="preserve">1=Family resources (parents, relatives, spouse, etc.) 2=Your own resources (income from work, work-study, etc.) 3=Aid that need not be repaid (grants, scholarships, military, etc.) 4=Aid that must be repaid (loans) 5=Other sources</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Financing education</t>
   </si>
   <si>
     <t xml:space="preserve">To what extent do you agree or disagree with the following statements? I am worried about my ability to pay for school. I am worried about my ability to repay my student loans in the future [if loans selected above] My student loans negatively impact my mental health [if loans selected above]</t>
@@ -4475,7 +4475,7 @@
       <c r="D15" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" s="2" t="s">
         <v>156</v>
       </c>
     </row>
@@ -4649,13 +4649,13 @@
         <v>427</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4663,7 +4663,7 @@
         <v>427</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>441</v>

</xml_diff>

<commit_message>
dry run fix #2
</commit_message>
<xml_diff>
--- a/SurveyQuestions/csvs/hms_survey.xlsx
+++ b/SurveyQuestions/csvs/hms_survey.xlsx
@@ -888,7 +888,7 @@
     <t xml:space="preserve">Display only if “Have you ever received counseling or therapy for mental health concerns?” is not “No, Never.”</t>
   </si>
   <si>
-    <t xml:space="preserve">How satisfied/dissatisfied are you with the following aspects of your therapy or counseling that you received in the past 12 months at [pipe in selected options from: “From which of the following places did you receive counseling or therapy?”]? Convenient hours Location [Do not display for digital resources] Quality of therapists/counselors Respect for my privacy concerns Ability to schedule appointments without long delays Respect and consideration for my identities (e.g., race/ethnicity, gender, etc.)</t>
+    <t xml:space="preserve">How satisfied/dissatisfied are you with the following aspects of your therapy or counseling that you received in the past 12 months at [pipe in selected options from: “From which of the following places did you receive counseling or therapy?”]? Convenient hours Location [Do not display for digital resources] Quality of therapists/counselors Respect for my privacy concerns Ability to schedule appointments without long delays Respect and consideration for my beliefs (e.g., faith, gender, etc.)</t>
   </si>
   <si>
     <t xml:space="preserve">Display only if "Have you ever received counseling or therapy for mental health concerns?" is not "No, Never." One matrix table question with 6 statements for each option selected for "From which of the following places did you receive counseling or therapy?" (Up to 8)</t>
@@ -1483,19 +1483,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4398,7 +4398,7 @@
       <c r="D10" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="1" t="s">
         <v>411</v>
       </c>
     </row>

</xml_diff>